<commit_message>
docs: add document pre-processing phase to task plan
</commit_message>
<xml_diff>
--- a/task_plan.xlsx
+++ b/task_plan.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,36 +458,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Architecture &amp; Foundation</t>
+          <t>Document Pre-processing</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Graph State Design</t>
+          <t>Document Loader Adapter</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Define `GraphState`, Pydantic schemas for node outputs.</t>
+          <t>Implement support for local/S3 file loading and Mime-type validation.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -500,86 +500,86 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Logprob Analyzer Engine</t>
+          <t>Page Splitting Logic</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Implement math logic for Margin calculation and confidence normalization.</t>
+          <t>Logic to split multi-page PDFs into individual images/sub-PDFs for processing.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OCR Integration Layer</t>
+          <t>Parallel OCR Orchestration</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Implement Azure DI wrapper with `ainvoke` support and error handling.</t>
+          <t>Implementation of concurrent page-level OCR using Azure DI.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Infrastructure Utilities</t>
+          <t>OCR Result Aggregator</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Setup Structlog, Pydantic-settings, and LangSmith tracing.</t>
+          <t>Merging page-level text, confidence, and metadata into a unified document object.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Base Unit Tests</t>
+          <t>Pre-processing Unit Tests</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Setup pytest for core utility functions (Logprob, OCR).</t>
+          <t>Validation of splitting, merging, and handling of corrupted/blurred files.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -592,140 +592,128 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Taxonomy &amp; Specialist Nodes</t>
+          <t>Architecture &amp; Foundation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>3.5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Root Router Implementation</t>
+          <t>Graph State Design</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Prompt engineering for MED vs NON classification.</t>
+          <t>Define `GraphState`, Pydantic schemas for node outputs.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medical Specialist (Sub-codes)</t>
+          <t>Logprob Analyzer Engine</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Implement medical node; Prompt tuning for LAB, CHK, OTH.</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>Implement math logic for Margin calculation and confidence normalization.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Non-Med Specialist (Sub-codes)</t>
+          <t>OCR Integration Layer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Implement non-med node; Prompt tuning for ID, PAS, OTH.</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>Implement Azure DI wrapper with `ainvoke` support and error handling.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pydantic Output Validation</t>
+          <t>Infrastructure Utilities</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Implement strict schema validation for LLM classification codes.</t>
+          <t>Setup Structlog, Pydantic-settings, and LangSmith tracing.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dynamic Taxonomy Config</t>
+          <t>Base Unit Tests</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Move class descriptions to JSON/YAML for non-code updates.</t>
+          <t>Setup pytest for core utility functions (Logprob, OCR).</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -738,36 +726,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Active Labeling Strategy</t>
+          <t>Taxonomy &amp; Specialist Nodes</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pilot Batch Processing</t>
+          <t>Root Router Implementation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Script to run 1,000+ docs through current pipeline; export data.</t>
+          <t>Prompt engineering for MED vs NON classification.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -780,40 +772,44 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verification Tooling</t>
+          <t>Medical Specialist (Sub-codes)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Build Streamlit UI for fast human verification (Image vs Prediction).</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>Implement medical node; Prompt tuning for LAB, CHK, OTH.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Human Labeling Execution</t>
+          <t>Non-Med Specialist (Sub-codes)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(External) Users verify predictions to create Gold Standard labels.</t>
+          <t>Implement non-med node; Prompt tuning for ID, PAS, OTH.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -830,245 +826,383 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ground Truth Sanitization</t>
+          <t>Pydantic Output Validation</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Script to resolve label conflicts and clean final evaluation set.</t>
+          <t>Implement strict schema validation for LLM classification codes.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Reliability Engineering</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+          <t>Dynamic Taxonomy Config</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Move class descriptions to JSON/YAML for non-code updates.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Confusion Matrix Analysis</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Evaluate against Gold Standard; find high False Positive classes.</t>
-        </is>
-      </c>
+          <t>Active Labeling Strategy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Margin Threshold Optimization</t>
+          <t>Pilot Batch Processing</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Plot precision/recall curves to find the optimal Margin Threshold.</t>
+          <t>Script to run 1,000+ docs through current pipeline; export data.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prompt Conflict Resolution</t>
+          <t>Verification Tooling</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Re-tune prompts to fix overlaps found during evaluation.</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+          <t>Build Streamlit UI for fast human verification (Image vs Prediction).</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Failure Case Documentation</t>
+          <t>Human Labeling Execution</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Create "Negative Examples" dataset for targeted performance tuning.</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>(External) Users verify predictions to create Gold Standard labels.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>API Layer &amp; Wrapper</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>Ground Truth Sanitization</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Script to resolve label conflicts and clean final evaluation set.</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FastAPI Endpoints</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>`/classify` (async), `/health`, and metadata endpoints.</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>Reliability Engineering</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>6.0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Validation Middleware</t>
+          <t>Confusion Matrix Analysis</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Input validation (File size, Mime type) and Global Exception Handling.</t>
+          <t>Evaluate against Gold Standard; find high False Positive classes.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Integration Docs</t>
+          <t>Margin Threshold Optimization</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Generate Swagger/Redoc and provide Client-side SDK samples.</t>
+          <t>Plot precision/recall curves to find the optimal Margin Threshold.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Prompt Conflict Resolution</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Re-tune prompts to fix overlaps found during evaluation.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Failure Case Documentation</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Create "Negative Examples" dataset for targeted performance tuning.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>API Layer &amp; Wrapper</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>FastAPI Endpoints</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>`/classify` (async), `/health`, and metadata endpoints.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Validation Middleware</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Input validation (File size, Mime type) and Global Exception Handling.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Integration Docs</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Generate Swagger/Redoc and provide Client-side SDK samples.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>23.0 MD</t>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>26.0 MD</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: replace dynamic config with node logic unit tests in task plan
</commit_message>
<xml_diff>
--- a/task_plan.xlsx
+++ b/task_plan.xlsx
@@ -854,12 +854,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dynamic Taxonomy Config</t>
+          <t>Node Logic Unit Tests</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Move class descriptions to JSON/YAML for non-code updates.</t>
+          <t>Unit tests with Mocked LLM responses to verify fallback logic and logprob extraction.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>

</xml_diff>